<commit_message>
Invest: keep the coming-soon page
Decision on 6 Oct: the Invest page stays "Coming soon" for now. The investor
access portal added in the previous commit is removed and the page is back to
the live version (only the stylesheet version differs).

The change workbook records it: the Invest row is marked undone (70 changes,
57 standing, 13 undone), the open item is marked decided, and the question for
counsel now asks whether "Coming soon" on the site is consistent with the
decks and teaser inviting investors through invest@nemilmm.com.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018MafBKjuv7rZ7cieL7GV7x
</commit_message>
<xml_diff>
--- a/_s4/NEMI_BCA-Ready_all_changes.xlsx
+++ b/_s4/NEMI_BCA-Ready_all_changes.xlsx
@@ -561,7 +561,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>5 Oct 2026. 70 changes. 58 make BCA-Ready differ from the live site (main); 12 were made and later undone, so that part now matches the live site again. Grey = live wording · Green = BCA-Ready wording · Blue status = undone. List # = item in the website update list.</t>
+          <t>6 Oct 2026. 70 changes. 57 make BCA-Ready differ from the live site (main); 13 were made and later undone, so that part now matches the live site again. Grey = live wording · Green = BCA-Ready wording · Blue status = undone. List # = item in the website update list. Checked against the plan, vPresent, vS, vShare, the Pre-IPO teaser, the Master Plan letter and the forecast.</t>
         </is>
       </c>
     </row>
@@ -4040,27 +4040,27 @@
       </c>
       <c r="E74" s="6" t="inlineStr">
         <is>
-          <t>Investor access portal: four steps (request access, sign the NDA, confirm accreditation, data room), a request form with email verification, investor type, country and indicative interest, two required confirmations (accredited or non-US; agrees to an NDA), and a securities legend. invest@nemilmm.com as an alternative.</t>
+          <t>Same as live: "Invest in NEMI — Coming soon. Our investment offerings are not open yet. Stay tuned."</t>
         </is>
       </c>
       <c r="F74" s="4" t="inlineStr">
         <is>
-          <t>"Coming soon" removed; the page now takes access requests. Requests arrive in the same inbox as contact enquiries, marked "INVESTOR ACCESS REQUEST".</t>
+          <t>A gated investor access portal was built on 5 Oct and removed on 6 Oct. The page stays "Coming soon".</t>
         </is>
       </c>
       <c r="G74" s="4" t="inlineStr">
         <is>
-          <t>The plan's option A: a gated portal. Nothing confidential is on the public page: no terms, valuation, projections or transaction. Materials go out only after NDA and accreditation. Still noindex.</t>
+          <t>Your decision on 6 Oct: keep the Invest page as "Coming soon" for now.</t>
         </is>
       </c>
       <c r="H74" s="4" t="inlineStr">
         <is>
-          <t>5 Oct</t>
-        </is>
-      </c>
-      <c r="I74" s="7" t="inlineStr">
-        <is>
-          <t>In BCA-Ready</t>
+          <t>5 Oct, undone 6 Oct</t>
+        </is>
+      </c>
+      <c r="I74" s="8" t="inlineStr">
+        <is>
+          <t>Undone · same as live</t>
         </is>
       </c>
       <c r="J74" s="4" t="inlineStr">
@@ -4263,52 +4263,52 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="6" t="n">
+      <c r="A7" s="5" t="n">
         <v>3</v>
       </c>
-      <c r="B7" s="7" t="inlineStr">
-        <is>
-          <t>Done 5 Oct</t>
-        </is>
-      </c>
-      <c r="C7" s="6" t="inlineStr">
+      <c r="B7" s="13" t="inlineStr">
+        <is>
+          <t>Decided 6 Oct</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
         <is>
           <t>Invest</t>
         </is>
       </c>
-      <c r="D7" s="6" t="inlineStr">
+      <c r="D7" s="5" t="inlineStr">
         <is>
           <t>Whole page</t>
         </is>
       </c>
-      <c r="E7" s="6" t="inlineStr">
+      <c r="E7" s="5" t="inlineStr">
         <is>
           <t>Invest in NEMI — Coming soon</t>
         </is>
       </c>
-      <c r="F7" s="6" t="inlineStr">
-        <is>
-          <t>Done 5 Oct: gated investor access portal live on BCA-Ready; "Coming soon" removed. Before launch: someone owns the inbox, the NDA template and the accreditation check (a third-party verification service or a letter from a CPA or attorney).</t>
-        </is>
-      </c>
-      <c r="G7" s="6" t="inlineStr">
+      <c r="F7" s="5" t="inlineStr">
+        <is>
+          <t>Decided 6 Oct: keep "Coming soon". The decks and teaser still invite investors through invest@nemilmm.com, and an investor site exists at invest-reg-d.nemilmm.com. Counsel to confirm the two are consistent (question drafted).</t>
+        </is>
+      </c>
+      <c r="G7" s="5" t="inlineStr">
         <is>
           <t>The teaser and decks send investors to invest@nemilmm.com; a public "coming soon" contradicts that.</t>
         </is>
       </c>
-      <c r="H7" s="6" t="inlineStr">
+      <c r="H7" s="5" t="inlineStr">
         <is>
           <t>CEO + counsel</t>
         </is>
       </c>
-      <c r="I7" s="6" t="inlineStr">
+      <c r="I7" s="5" t="inlineStr">
         <is>
           <t>23</t>
         </is>
       </c>
-      <c r="J7" s="6" t="inlineStr">
-        <is>
-          <t>Done</t>
+      <c r="J7" s="5" t="inlineStr">
+        <is>
+          <t>Not needed</t>
         </is>
       </c>
     </row>
@@ -5578,7 +5578,7 @@
           <t>1. Our pre-NDA investor teaser describes the transaction process with dates. Can a pre-NDA document carry that before announcement, or should it come out?
 2. The website footer now reads "© 2026 NEMI Corp." Please confirm the exact legal name the S-4 will use.
 3. The founder's letter on the website says "MaaS is profitable on its own" and "profitably, today". The group is not profitable; the MaaS segment is EBITDA-positive on management figures. Should the letter state the segment measure, or should the lines come out?
-4. We have opened a gated investor access page (request, NDA, accreditation check, data room). Please review the page wording and the legend.
+4. The website's Invest page says "Coming soon", while our decks and teaser invite investors through invest@nemilmm.com, and an investor site exists at invest-reg-d.nemilmm.com. Is that consistent, or should one of them change?
 5. Two advisors and a director may need relationship disclosures. Please advise what the S-4 requires.</t>
         </is>
       </c>

</xml_diff>

<commit_message>
About: team cards follow vShare and vPresent
Decision on 6 Oct: the October decks are the source of truth for facts. Every
team card now carries the deck wording: the CEO's "built NEMI greenfield to
300k sq ft", Kevin Flick's principal-investing bio, Mary Pruce's RK Pharma
bio, Jingjing Kanik's CVS Health bio, "Board Advisor" and "Advisor" titles,
and Subramanian Ramasamy as Chief Financial Officer · India. Gokul Madhavan's
bio is the deck's, including his A.B. The page notes that called the Kevin and
Gokul bios interim are removed.

The change workbook: every done or decided item now sits on "All changes"
(83 rows: 50 in place, 20 undone, 13 checked and kept against the decks).
"Still to update" holds only the Invest page. The drafted-messages tab is
gone, as each question was settled from the decks.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018MafBKjuv7rZ7cieL7GV7x
</commit_message>
<xml_diff>
--- a/_s4/NEMI_BCA-Ready_all_changes.xlsx
+++ b/_s4/NEMI_BCA-Ready_all_changes.xlsx
@@ -9,11 +9,10 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="All changes" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Still to update" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Messages to send" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'All changes'!$A$4:$J$74</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Still to update'!$A$4:$J$33</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'All changes'!$A$4:$J$87</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Still to update'!$A$4:$J$5</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -536,7 +535,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J74"/>
+  <dimension ref="A1:J87"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -561,7 +560,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>6 Oct 2026. 70 changes. 57 make BCA-Ready differ from the live site (main); 13 were made and later undone, so that part now matches the live site again. Grey = live wording · Green = BCA-Ready wording · Blue status = undone. List # = item in the website update list. Checked against the plan, vPresent, vS, vShare, the Pre-IPO teaser, the Master Plan letter and the forecast.</t>
+          <t>6 Oct 2026. 83 rows, everything done or decided to date. 50 make BCA-Ready differ from the live site; 20 were made and later undone, so that part matches the live site again; 13 were checked and kept as they are. Source of truth for facts: vShare and vPresent (Oct 2026). Grey = live wording · Green = BCA-Ready wording. List # = item in the website update list.</t>
         </is>
       </c>
     </row>
@@ -1480,27 +1479,27 @@
       </c>
       <c r="E22" s="6" t="inlineStr">
         <is>
-          <t>Built NEMI's EV business and acquired and expanded its MaaS factories, now over 300,000 sq ft in India.</t>
+          <t>Same as live: "…Built NEMI greenfield to 300k sq ft." (Director card: no footprint line)</t>
         </is>
       </c>
       <c r="F22" s="4" t="inlineStr">
         <is>
-          <t>"Greenfield" replaced with the history the letter describes: EV business built in-house, MaaS factories acquired and expanded.</t>
+          <t>Changed twice before 6 Oct ("acquired and expanded…", then "built the EV business and acquired…"); back to the deck wording on 6 Oct.</t>
         </is>
       </c>
       <c r="G22" s="4" t="inlineStr">
         <is>
-          <t>The letter: capabilities were built on NEMI's own EV business; the MaaS business came from an acquisition 2 years ago. The decks were corrected to match (copies sent separately, not in this repo).</t>
+          <t>Source of truth: vShare and vPresent (Oct 2026). Both say "built NEMI greenfield to 300k sq ft" (vShare slide 11, vPresent slide 21).</t>
         </is>
       </c>
       <c r="H22" s="4" t="inlineStr">
         <is>
-          <t>Before 5 Oct, rewritten 5 Oct</t>
-        </is>
-      </c>
-      <c r="I22" s="7" t="inlineStr">
-        <is>
-          <t>In BCA-Ready</t>
+          <t>Before 5 Oct, undone 6 Oct</t>
+        </is>
+      </c>
+      <c r="I22" s="8" t="inlineStr">
+        <is>
+          <t>Undone · same as live</t>
         </is>
       </c>
       <c r="J22" s="4" t="inlineStr">
@@ -1530,27 +1529,27 @@
       </c>
       <c r="E23" s="6" t="inlineStr">
         <is>
-          <t>Two decades in senior finance roles across energy and industrial businesses, including a decade at Canacol Energy and transaction advisory at EY.</t>
+          <t>Same as live: "20+ years in principal investing, capital markets and M&amp;A. $5B+ raised, three listings on NASDAQ, NYSE and TSX. Goldman Sachs, Hicks Muse, EY."</t>
         </is>
       </c>
       <c r="F23" s="4" t="inlineStr">
         <is>
-          <t>General bio written from his LinkedIn.</t>
+          <t>The LinkedIn-based bio is replaced by the deck bio.</t>
         </is>
       </c>
       <c r="G23" s="4" t="inlineStr">
         <is>
-          <t>Goldman Sachs and Hicks Muse do not appear in his LinkedIn history. Must be checked against his CV and match the S-4 before filing.</t>
+          <t>Source of truth: vShare and vPresent (Oct 2026). Both carry this bio word for word.</t>
         </is>
       </c>
       <c r="H23" s="4" t="inlineStr">
         <is>
-          <t>Before 5 Oct</t>
-        </is>
-      </c>
-      <c r="I23" s="7" t="inlineStr">
-        <is>
-          <t>In BCA-Ready</t>
+          <t>Before 5 Oct, undone 6 Oct</t>
+        </is>
+      </c>
+      <c r="I23" s="8" t="inlineStr">
+        <is>
+          <t>Undone · same as live</t>
         </is>
       </c>
       <c r="J23" s="4" t="inlineStr">
@@ -1580,27 +1579,27 @@
       </c>
       <c r="E24" s="6" t="inlineStr">
         <is>
-          <t>Two decades building people functions in healthcare and pharma. Head of HR at RK Pharma, chief people officer at InTouch Med Supply. SHRM-SCP and SPHR certified.</t>
+          <t>Same as live.</t>
         </is>
       </c>
       <c r="F24" s="4" t="inlineStr">
         <is>
-          <t>Fuller bio.</t>
+          <t>Fuller bio replaced by the deck bio.</t>
         </is>
       </c>
       <c r="G24" s="4" t="inlineStr">
         <is>
-          <t>Updated bio.</t>
+          <t>Source of truth: vShare and vPresent (Oct 2026). "Senior HR executive; most recently Head of Human Resources at RK Pharma Inc. SHRM-SCP · HRCI-SPHR".</t>
         </is>
       </c>
       <c r="H24" s="4" t="inlineStr">
         <is>
-          <t>Before 5 Oct</t>
-        </is>
-      </c>
-      <c r="I24" s="7" t="inlineStr">
-        <is>
-          <t>In BCA-Ready</t>
+          <t>Before 5 Oct, undone 6 Oct</t>
+        </is>
+      </c>
+      <c r="I24" s="8" t="inlineStr">
+        <is>
+          <t>Undone · same as live</t>
         </is>
       </c>
       <c r="J24" s="4" t="inlineStr"/>
@@ -1626,22 +1625,22 @@
       </c>
       <c r="E25" s="6" t="inlineStr">
         <is>
-          <t>Corporate development and transformation. M&amp;A integration, digital finance operations, and the work of turning strategy into operating plans across the group. PhD Harvard, MBA Yale.</t>
+          <t>Led M&amp;A integrations, built digital finance operations and led digital transformations. A.B. and PhD Harvard, MBA Yale.</t>
         </is>
       </c>
       <c r="F25" s="4" t="inlineStr">
         <is>
-          <t>Reframed for the strategy title. Degrees were cut before 5 Oct and put back on 5 Oct.</t>
+          <t>Interim strategy wording replaced by the deck bio, including his A.B.</t>
         </is>
       </c>
       <c r="G25" s="4" t="inlineStr">
         <is>
-          <t>Interim wording until he sends his own; degrees are in every deck.</t>
+          <t>Source of truth: vShare and vPresent (Oct 2026). "Led M&amp;A integrations, built digital finance ops, led digital transformations. A.B. + PhD Harvard · MBA Yale".</t>
         </is>
       </c>
       <c r="H25" s="4" t="inlineStr">
         <is>
-          <t>Before 5 Oct, corrected 5 Oct</t>
+          <t>Before 5 Oct, settled 6 Oct</t>
         </is>
       </c>
       <c r="I25" s="7" t="inlineStr">
@@ -1864,22 +1863,22 @@
       </c>
       <c r="E30" s="6" t="inlineStr">
         <is>
-          <t>Finance Head · India (code FIN). Bio same as live.</t>
+          <t>Chief Financial Officer · India (code CFO). Name: Subramanian Ramasamy. Bio same as live.</t>
         </is>
       </c>
       <c r="F30" s="4" t="inlineStr">
         <is>
-          <t>Title changed. A bio line added before 5 Oct ("Greenfield project expert") was removed on 5 Oct.</t>
+          <t>Title back to CFO · India (it had been "Finance Head · India"); name spelt as the decks spell it.</t>
         </is>
       </c>
       <c r="G30" s="4" t="inlineStr">
         <is>
-          <t>Two CFOs on one page would confuse the S-4 officer list. The decks still say "CFO · India": align them.</t>
+          <t>Source of truth: vShare and vPresent (Oct 2026). vPresent slide 22: "Subramanian Ramasamy · CFO · India".</t>
         </is>
       </c>
       <c r="H30" s="4" t="inlineStr">
         <is>
-          <t>Before 5 Oct, corrected 5 Oct</t>
+          <t>Before 5 Oct, settled 6 Oct</t>
         </is>
       </c>
       <c r="I30" s="7" t="inlineStr">
@@ -2056,27 +2055,27 @@
       </c>
       <c r="E34" s="6" t="inlineStr">
         <is>
-          <t>Data and AI leader in aerospace and healthcare. VP of integrated business planning at Pursuit Aerospace, previously Executive Director of Data Science at CVS Health. Ex-McKinsey. PhD, Yale.</t>
+          <t>Same as live: "Executive Director of Data Science at CVS Health, ex-McKinsey. PhD, Yale."</t>
         </is>
       </c>
       <c r="F34" s="4" t="inlineStr">
         <is>
-          <t>Current role at Pursuit Aerospace added; deck facts kept.</t>
+          <t>Pursuit Aerospace line removed.</t>
         </is>
       </c>
       <c r="G34" s="4" t="inlineStr">
         <is>
-          <t>Newer role. Needs her sign-off and must match the S-4.</t>
+          <t>Source of truth: vShare and vPresent (Oct 2026). vPresent slide 22.</t>
         </is>
       </c>
       <c r="H34" s="4" t="inlineStr">
         <is>
-          <t>Before 5 Oct, corrected 5 Oct</t>
-        </is>
-      </c>
-      <c r="I34" s="7" t="inlineStr">
-        <is>
-          <t>In BCA-Ready</t>
+          <t>Before 5 Oct, undone 6 Oct</t>
+        </is>
+      </c>
+      <c r="I34" s="8" t="inlineStr">
+        <is>
+          <t>Undone · same as live</t>
         </is>
       </c>
       <c r="J34" s="4" t="inlineStr"/>
@@ -2198,27 +2197,27 @@
       </c>
       <c r="E37" s="6" t="inlineStr">
         <is>
-          <t>Chairman · AxisCades. Bio same as live.</t>
+          <t>Same as live: Board Advisor · Chairman and MD of AXISCADES…</t>
         </is>
       </c>
       <c r="F37" s="4" t="inlineStr">
         <is>
-          <t>Title changed. Name was spelt "Ravinarayanan" and "Founder of Microcon" added; both undone on 5 Oct.</t>
+          <t>Title back to "Board Advisor".</t>
         </is>
       </c>
       <c r="G37" s="4" t="inlineStr">
         <is>
-          <t>Every document spells it as two words; Microcon is in no document.</t>
+          <t>Source of truth: vShare and vPresent (Oct 2026). vPresent slide 22: "Board Advisor".</t>
         </is>
       </c>
       <c r="H37" s="4" t="inlineStr">
         <is>
-          <t>Before 5 Oct, corrected 5 Oct</t>
-        </is>
-      </c>
-      <c r="I37" s="7" t="inlineStr">
-        <is>
-          <t>In BCA-Ready</t>
+          <t>Before 5 Oct, undone 6 Oct</t>
+        </is>
+      </c>
+      <c r="I37" s="8" t="inlineStr">
+        <is>
+          <t>Undone · same as live</t>
         </is>
       </c>
       <c r="J37" s="4" t="inlineStr">
@@ -2248,27 +2247,27 @@
       </c>
       <c r="E38" s="6" t="inlineStr">
         <is>
-          <t>Ex-CEO · Ashok Leyland. Bio same as live.</t>
+          <t>Same as live: Advisor · Former MD and CEO of Ashok Leyland and Royal Enfield.</t>
         </is>
       </c>
       <c r="F38" s="4" t="inlineStr">
         <is>
-          <t>Title shows his former role. An added line was removed on 5 Oct.</t>
+          <t>Title back to "Advisor".</t>
         </is>
       </c>
       <c r="G38" s="4" t="inlineStr">
         <is>
-          <t>Clearer title; unsourced addition removed.</t>
+          <t>Source of truth: vShare and vPresent (Oct 2026). vPresent slide 22: "Advisor".</t>
         </is>
       </c>
       <c r="H38" s="4" t="inlineStr">
         <is>
-          <t>Before 5 Oct, corrected 5 Oct</t>
-        </is>
-      </c>
-      <c r="I38" s="7" t="inlineStr">
-        <is>
-          <t>In BCA-Ready</t>
+          <t>Before 5 Oct, undone 6 Oct</t>
+        </is>
+      </c>
+      <c r="I38" s="8" t="inlineStr">
+        <is>
+          <t>Undone · same as live</t>
         </is>
       </c>
       <c r="J38" s="4" t="inlineStr">
@@ -2298,27 +2297,27 @@
       </c>
       <c r="E39" s="6" t="inlineStr">
         <is>
-          <t>Ex-Sr Partner · McKinsey · Senior Partner Emeritus, McKinsey &amp; Company (30 years). Former head of McKinsey's Industrial practice in South Asia.</t>
+          <t>Same as live: Advisor · Senior Partner Emeritus at McKinsey &amp; Company, 30 years.</t>
         </is>
       </c>
       <c r="F39" s="4" t="inlineStr">
         <is>
-          <t>Title and one line, in the decks' wording.</t>
+          <t>Title back to "Advisor"; added line removed.</t>
         </is>
       </c>
       <c r="G39" s="4" t="inlineStr">
         <is>
-          <t>vPresent: "ex-McKinsey, Industrial South Asia head".</t>
+          <t>Source of truth: vShare and vPresent (Oct 2026). vPresent slide 22: "Advisor · Senior Partner Emeritus, McKinsey (30 yrs)".</t>
         </is>
       </c>
       <c r="H39" s="4" t="inlineStr">
         <is>
-          <t>Before 5 Oct, corrected 5 Oct</t>
-        </is>
-      </c>
-      <c r="I39" s="7" t="inlineStr">
-        <is>
-          <t>In BCA-Ready</t>
+          <t>Before 5 Oct, undone 6 Oct</t>
+        </is>
+      </c>
+      <c r="I39" s="8" t="inlineStr">
+        <is>
+          <t>Undone · same as live</t>
         </is>
       </c>
       <c r="J39" s="4" t="inlineStr">
@@ -3058,12 +3057,12 @@
       </c>
       <c r="G54" s="4" t="inlineStr">
         <is>
-          <t>Benchmark not in any company document. Under $0.5M is the figure every deck uses. CFO to confirm against the ledger.</t>
+          <t>Benchmark not in any company document. Source of truth: vShare and vPresent (Oct 2026). Both say "under $0.5M".</t>
         </is>
       </c>
       <c r="H54" s="4" t="inlineStr">
         <is>
-          <t>Before 5 Oct, updated 5 Oct</t>
+          <t>Before 5 Oct, settled 6 Oct</t>
         </is>
       </c>
       <c r="I54" s="7" t="inlineStr">
@@ -4069,8 +4068,606 @@
         </is>
       </c>
     </row>
+    <row r="75">
+      <c r="A75" s="4" t="n">
+        <v>71</v>
+      </c>
+      <c r="B75" s="4" t="inlineStr">
+        <is>
+          <t>Case Messenger (BNC)</t>
+        </is>
+      </c>
+      <c r="C75" s="4" t="inlineStr">
+        <is>
+          <t>Results: 9 months, 50% compression, 100% spec met, sub-$1,000</t>
+        </is>
+      </c>
+      <c r="D75" s="5" t="inlineStr">
+        <is>
+          <t>As on the site</t>
+        </is>
+      </c>
+      <c r="E75" s="6" t="inlineStr">
+        <is>
+          <t>Same</t>
+        </is>
+      </c>
+      <c r="F75" s="4" t="inlineStr">
+        <is>
+          <t>Kept.</t>
+        </is>
+      </c>
+      <c r="G75" s="4" t="inlineStr">
+        <is>
+          <t>Source of truth: vShare and vPresent (Oct 2026). "Full EV platform in 9 months, under $0.5M". The site matches; the other figures stay as published.</t>
+        </is>
+      </c>
+      <c r="H75" s="4" t="inlineStr">
+        <is>
+          <t>6 Oct</t>
+        </is>
+      </c>
+      <c r="I75" s="11" t="inlineStr">
+        <is>
+          <t>Decided · no website change</t>
+        </is>
+      </c>
+      <c r="J75" s="4" t="inlineStr"/>
+    </row>
+    <row r="76">
+      <c r="A76" s="4" t="n">
+        <v>72</v>
+      </c>
+      <c r="B76" s="4" t="inlineStr">
+        <is>
+          <t>Case Coffee</t>
+        </is>
+      </c>
+      <c r="C76" s="4" t="inlineStr">
+        <is>
+          <t>Results: 12+ to 5 weeks, ~$100k, −20% BOM, 400 a month</t>
+        </is>
+      </c>
+      <c r="D76" s="5" t="inlineStr">
+        <is>
+          <t>As on the site</t>
+        </is>
+      </c>
+      <c r="E76" s="6" t="inlineStr">
+        <is>
+          <t>Same</t>
+        </is>
+      </c>
+      <c r="F76" s="4" t="inlineStr">
+        <is>
+          <t>Kept.</t>
+        </is>
+      </c>
+      <c r="G76" s="4" t="inlineStr">
+        <is>
+          <t>Source of truth: vShare and vPresent (Oct 2026). The decks cite this customer ("our single most important vendor partner") and hold the full case in the data room.</t>
+        </is>
+      </c>
+      <c r="H76" s="4" t="inlineStr">
+        <is>
+          <t>6 Oct</t>
+        </is>
+      </c>
+      <c r="I76" s="11" t="inlineStr">
+        <is>
+          <t>Decided · no website change</t>
+        </is>
+      </c>
+      <c r="J76" s="4" t="inlineStr"/>
+    </row>
+    <row r="77">
+      <c r="A77" s="4" t="n">
+        <v>73</v>
+      </c>
+      <c r="B77" s="4" t="inlineStr">
+        <is>
+          <t>Case Drone · Case Studies</t>
+        </is>
+      </c>
+      <c r="C77" s="4" t="inlineStr">
+        <is>
+          <t>Results: 16 to 4 months, $100k, 4/4 in-house, −20% BOM, 4× faster</t>
+        </is>
+      </c>
+      <c r="D77" s="5" t="inlineStr">
+        <is>
+          <t>As on the site</t>
+        </is>
+      </c>
+      <c r="E77" s="6" t="inlineStr">
+        <is>
+          <t>Same</t>
+        </is>
+      </c>
+      <c r="F77" s="4" t="inlineStr">
+        <is>
+          <t>Kept.</t>
+        </is>
+      </c>
+      <c r="G77" s="4" t="inlineStr">
+        <is>
+          <t>Source of truth: vShare and vPresent (Oct 2026). "Full drone powertrain in 4 months vs 16-month benchmark · 4× faster · −20% BOM · all four components in-house".</t>
+        </is>
+      </c>
+      <c r="H77" s="4" t="inlineStr">
+        <is>
+          <t>6 Oct</t>
+        </is>
+      </c>
+      <c r="I77" s="11" t="inlineStr">
+        <is>
+          <t>Decided · no website change</t>
+        </is>
+      </c>
+      <c r="J77" s="4" t="inlineStr"/>
+    </row>
+    <row r="78">
+      <c r="A78" s="4" t="n">
+        <v>74</v>
+      </c>
+      <c r="B78" s="4" t="inlineStr">
+        <is>
+          <t>Case PMI · Case Studies</t>
+        </is>
+      </c>
+      <c r="C78" s="4" t="inlineStr">
+        <is>
+          <t>Results: 7 to 3 hrs, ~15 a day, 10–15 µm, under a week</t>
+        </is>
+      </c>
+      <c r="D78" s="5" t="inlineStr">
+        <is>
+          <t>As on the site</t>
+        </is>
+      </c>
+      <c r="E78" s="6" t="inlineStr">
+        <is>
+          <t>Same</t>
+        </is>
+      </c>
+      <c r="F78" s="4" t="inlineStr">
+        <is>
+          <t>Kept.</t>
+        </is>
+      </c>
+      <c r="G78" s="4" t="inlineStr">
+        <is>
+          <t>Source of truth: vShare and vPresent (Oct 2026). "Flight-critical clamp held to 10–15 μm, supplied in days".</t>
+        </is>
+      </c>
+      <c r="H78" s="4" t="inlineStr">
+        <is>
+          <t>6 Oct</t>
+        </is>
+      </c>
+      <c r="I78" s="11" t="inlineStr">
+        <is>
+          <t>Decided · no website change</t>
+        </is>
+      </c>
+      <c r="J78" s="4" t="inlineStr"/>
+    </row>
+    <row r="79">
+      <c r="A79" s="4" t="n">
+        <v>75</v>
+      </c>
+      <c r="B79" s="4" t="inlineStr">
+        <is>
+          <t>Case Drone</t>
+        </is>
+      </c>
+      <c r="C79" s="4" t="inlineStr">
+        <is>
+          <t>Hero image</t>
+        </is>
+      </c>
+      <c r="D79" s="5" t="inlineStr">
+        <is>
+          <t>Labelled "Illustration. Not the delivered airframe."</t>
+        </is>
+      </c>
+      <c r="E79" s="6" t="inlineStr">
+        <is>
+          <t>Same</t>
+        </is>
+      </c>
+      <c r="F79" s="4" t="inlineStr">
+        <is>
+          <t>Kept with the label.</t>
+        </is>
+      </c>
+      <c r="G79" s="4" t="inlineStr">
+        <is>
+          <t>The label already says it is not the customer's airframe.</t>
+        </is>
+      </c>
+      <c r="H79" s="4" t="inlineStr">
+        <is>
+          <t>6 Oct</t>
+        </is>
+      </c>
+      <c r="I79" s="11" t="inlineStr">
+        <is>
+          <t>Decided · no website change</t>
+        </is>
+      </c>
+      <c r="J79" s="4" t="inlineStr"/>
+    </row>
+    <row r="80">
+      <c r="A80" s="4" t="n">
+        <v>76</v>
+      </c>
+      <c r="B80" s="4" t="inlineStr">
+        <is>
+          <t>FAQ · footer badges</t>
+        </is>
+      </c>
+      <c r="C80" s="4" t="inlineStr">
+        <is>
+          <t>Certifications</t>
+        </is>
+      </c>
+      <c r="D80" s="5" t="inlineStr">
+        <is>
+          <t>AS9100D:2016 and ISO 9001:2015</t>
+        </is>
+      </c>
+      <c r="E80" s="6" t="inlineStr">
+        <is>
+          <t>Same</t>
+        </is>
+      </c>
+      <c r="F80" s="4" t="inlineStr">
+        <is>
+          <t>Kept.</t>
+        </is>
+      </c>
+      <c r="G80" s="4" t="inlineStr">
+        <is>
+          <t>Source of truth: vShare and vPresent (Oct 2026). "AS9100D:2016 / ISO 9001:2015 / Certified".</t>
+        </is>
+      </c>
+      <c r="H80" s="4" t="inlineStr">
+        <is>
+          <t>6 Oct</t>
+        </is>
+      </c>
+      <c r="I80" s="11" t="inlineStr">
+        <is>
+          <t>Decided · no website change</t>
+        </is>
+      </c>
+      <c r="J80" s="4" t="inlineStr"/>
+    </row>
+    <row r="81">
+      <c r="A81" s="4" t="n">
+        <v>77</v>
+      </c>
+      <c r="B81" s="4" t="inlineStr">
+        <is>
+          <t>Home</t>
+        </is>
+      </c>
+      <c r="C81" s="4" t="inlineStr">
+        <is>
+          <t>App screenshots (Anvil, Orion, Atlas)</t>
+        </is>
+      </c>
+      <c r="D81" s="5" t="inlineStr">
+        <is>
+          <t>Screens with status badges</t>
+        </is>
+      </c>
+      <c r="E81" s="6" t="inlineStr">
+        <is>
+          <t>Same</t>
+        </is>
+      </c>
+      <c r="F81" s="4" t="inlineStr">
+        <is>
+          <t>Kept.</t>
+        </is>
+      </c>
+      <c r="G81" s="4" t="inlineStr">
+        <is>
+          <t>Source of truth: vShare and vPresent (Oct 2026). vPresent slide 7: "Live screens, not mockups".</t>
+        </is>
+      </c>
+      <c r="H81" s="4" t="inlineStr">
+        <is>
+          <t>6 Oct</t>
+        </is>
+      </c>
+      <c r="I81" s="11" t="inlineStr">
+        <is>
+          <t>Decided · no website change</t>
+        </is>
+      </c>
+      <c r="J81" s="4" t="inlineStr"/>
+    </row>
+    <row r="82">
+      <c r="A82" s="4" t="n">
+        <v>78</v>
+      </c>
+      <c r="B82" s="4" t="inlineStr">
+        <is>
+          <t>Home</t>
+        </is>
+      </c>
+      <c r="C82" s="4" t="inlineStr">
+        <is>
+          <t>Market images and BOSS E-TWIN</t>
+        </is>
+      </c>
+      <c r="D82" s="5" t="inlineStr">
+        <is>
+          <t>Market photos under "The Markets We Build For"</t>
+        </is>
+      </c>
+      <c r="E82" s="6" t="inlineStr">
+        <is>
+          <t>Same</t>
+        </is>
+      </c>
+      <c r="F82" s="4" t="inlineStr">
+        <is>
+          <t>Kept.</t>
+        </is>
+      </c>
+      <c r="G82" s="4" t="inlineStr">
+        <is>
+          <t>Source of truth: vShare and vPresent (Oct 2026). The heading presents them as target markets; the decks show work across NEMI group entities.</t>
+        </is>
+      </c>
+      <c r="H82" s="4" t="inlineStr">
+        <is>
+          <t>6 Oct</t>
+        </is>
+      </c>
+      <c r="I82" s="11" t="inlineStr">
+        <is>
+          <t>Decided · no website change</t>
+        </is>
+      </c>
+      <c r="J82" s="4" t="inlineStr"/>
+    </row>
+    <row r="83">
+      <c r="A83" s="4" t="n">
+        <v>79</v>
+      </c>
+      <c r="B83" s="4" t="inlineStr">
+        <is>
+          <t>About · Home · Offerings</t>
+        </is>
+      </c>
+      <c r="C83" s="4" t="inlineStr">
+        <is>
+          <t>Archive photos and videos</t>
+        </is>
+      </c>
+      <c r="D83" s="5" t="inlineStr">
+        <is>
+          <t>As on the site</t>
+        </is>
+      </c>
+      <c r="E83" s="6" t="inlineStr">
+        <is>
+          <t>Same</t>
+        </is>
+      </c>
+      <c r="F83" s="4" t="inlineStr">
+        <is>
+          <t>Kept.</t>
+        </is>
+      </c>
+      <c r="G83" s="4" t="inlineStr">
+        <is>
+          <t>Published on the live site; no deck content conflicts.</t>
+        </is>
+      </c>
+      <c r="H83" s="4" t="inlineStr">
+        <is>
+          <t>6 Oct</t>
+        </is>
+      </c>
+      <c r="I83" s="11" t="inlineStr">
+        <is>
+          <t>Decided · no website change</t>
+        </is>
+      </c>
+      <c r="J83" s="4" t="inlineStr"/>
+    </row>
+    <row r="84">
+      <c r="A84" s="4" t="n">
+        <v>80</v>
+      </c>
+      <c r="B84" s="4" t="inlineStr">
+        <is>
+          <t>Teaser (pre-NDA)</t>
+        </is>
+      </c>
+      <c r="C84" s="4" t="inlineStr">
+        <is>
+          <t>Path-to-listing section</t>
+        </is>
+      </c>
+      <c r="D84" s="5" t="inlineStr">
+        <is>
+          <t>Not on the website</t>
+        </is>
+      </c>
+      <c r="E84" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F84" s="4" t="inlineStr">
+        <is>
+          <t>No website change.</t>
+        </is>
+      </c>
+      <c r="G84" s="4" t="inlineStr">
+        <is>
+          <t>The teaser is not part of the website.</t>
+        </is>
+      </c>
+      <c r="H84" s="4" t="inlineStr">
+        <is>
+          <t>6 Oct</t>
+        </is>
+      </c>
+      <c r="I84" s="11" t="inlineStr">
+        <is>
+          <t>Decided · no website change</t>
+        </is>
+      </c>
+      <c r="J84" s="4" t="inlineStr"/>
+    </row>
+    <row r="85">
+      <c r="A85" s="4" t="n">
+        <v>81</v>
+      </c>
+      <c r="B85" s="4" t="inlineStr">
+        <is>
+          <t>Decks and teaser</t>
+        </is>
+      </c>
+      <c r="C85" s="4" t="inlineStr">
+        <is>
+          <t>Customer count, retention, productivity</t>
+        </is>
+      </c>
+      <c r="D85" s="5" t="inlineStr">
+        <is>
+          <t>Not on the website</t>
+        </is>
+      </c>
+      <c r="E85" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F85" s="4" t="inlineStr">
+        <is>
+          <t>No website change.</t>
+        </is>
+      </c>
+      <c r="G85" s="4" t="inlineStr">
+        <is>
+          <t>The site does not carry these figures; the decks remain the source.</t>
+        </is>
+      </c>
+      <c r="H85" s="4" t="inlineStr">
+        <is>
+          <t>6 Oct</t>
+        </is>
+      </c>
+      <c r="I85" s="11" t="inlineStr">
+        <is>
+          <t>Decided · no website change</t>
+        </is>
+      </c>
+      <c r="J85" s="4" t="inlineStr"/>
+    </row>
+    <row r="86">
+      <c r="A86" s="4" t="n">
+        <v>82</v>
+      </c>
+      <c r="B86" s="4" t="inlineStr">
+        <is>
+          <t>LMM Stack · About</t>
+        </is>
+      </c>
+      <c r="C86" s="4" t="inlineStr">
+        <is>
+          <t>Footprint note "expansion planned"</t>
+        </is>
+      </c>
+      <c r="D86" s="5" t="inlineStr">
+        <is>
+          <t>Not added</t>
+        </is>
+      </c>
+      <c r="E86" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F86" s="4" t="inlineStr">
+        <is>
+          <t>Not added.</t>
+        </is>
+      </c>
+      <c r="G86" s="4" t="inlineStr">
+        <is>
+          <t>A forward-looking line; "more locations coming soon" was removed for the same reason.</t>
+        </is>
+      </c>
+      <c r="H86" s="4" t="inlineStr">
+        <is>
+          <t>6 Oct</t>
+        </is>
+      </c>
+      <c r="I86" s="11" t="inlineStr">
+        <is>
+          <t>Decided · no website change</t>
+        </is>
+      </c>
+      <c r="J86" s="4" t="inlineStr"/>
+    </row>
+    <row r="87">
+      <c r="A87" s="4" t="n">
+        <v>83</v>
+      </c>
+      <c r="B87" s="4" t="inlineStr">
+        <is>
+          <t>About · Master Plan</t>
+        </is>
+      </c>
+      <c r="C87" s="4" t="inlineStr">
+        <is>
+          <t>Phase names in the deck's words</t>
+        </is>
+      </c>
+      <c r="D87" s="5" t="inlineStr">
+        <is>
+          <t>Not changed</t>
+        </is>
+      </c>
+      <c r="E87" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F87" s="4" t="inlineStr">
+        <is>
+          <t>Not changed.</t>
+        </is>
+      </c>
+      <c r="G87" s="4" t="inlineStr">
+        <is>
+          <t>The founder's letter keeps its own wording, as published.</t>
+        </is>
+      </c>
+      <c r="H87" s="4" t="inlineStr">
+        <is>
+          <t>6 Oct</t>
+        </is>
+      </c>
+      <c r="I87" s="11" t="inlineStr">
+        <is>
+          <t>Decided · no website change</t>
+        </is>
+      </c>
+      <c r="J87" s="4" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:J74"/>
+  <autoFilter ref="A4:J87"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -4081,7 +4678,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J33"/>
+  <dimension ref="A1:J5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -4106,7 +4703,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Open items first. 1 · Decide = a person must choose before signing. 2 · Decide = before filing. 3 · Evidence = a document on file or the claim comes down. Done and not-needed items are marked green or grey.</t>
+          <t>One item left. Everything else is done or decided and listed on "All changes".</t>
         </is>
       </c>
     </row>
@@ -4163,1337 +4760,57 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="6" t="n">
+      <c r="A5" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="B5" s="7" t="inlineStr">
-        <is>
-          <t>Done 5 Oct</t>
-        </is>
-      </c>
-      <c r="C5" s="6" t="inlineStr">
-        <is>
-          <t>Master Plan</t>
-        </is>
-      </c>
-      <c r="D5" s="6" t="inlineStr">
-        <is>
-          <t>Founder's letter</t>
-        </is>
-      </c>
-      <c r="E5" s="6" t="inlineStr">
-        <is>
-          <t>Latest letter (Sep 2026) on both the Master Plan page and About, word for word. No forward-looking note.</t>
-        </is>
-      </c>
-      <c r="F5" s="6" t="inlineStr">
-        <is>
-          <t>Decided: publish the letter as written. For counsel before filing: the plan flags "The only way", the cellphone line, "MaaS is profitable on its own" and "profitably, today".</t>
-        </is>
-      </c>
-      <c r="G5" s="6" t="inlineStr">
-        <is>
-          <t>The plan flags these as High risk; two versions of one letter on one site is its own problem.</t>
-        </is>
-      </c>
-      <c r="H5" s="6" t="inlineStr">
-        <is>
-          <t>CEO + counsel</t>
-        </is>
-      </c>
-      <c r="I5" s="6" t="inlineStr">
-        <is>
-          <t>4, 5</t>
-        </is>
-      </c>
-      <c r="J5" s="6" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="B6" s="7" t="inlineStr">
-        <is>
-          <t>Done 5 Oct</t>
-        </is>
-      </c>
-      <c r="C6" s="6" t="inlineStr">
-        <is>
-          <t>All pages</t>
-        </is>
-      </c>
-      <c r="D6" s="6" t="inlineStr">
-        <is>
-          <t>Footer</t>
-        </is>
-      </c>
-      <c r="E6" s="6" t="inlineStr">
-        <is>
-          <t>© 2026 NEMI Corp. All rights reserved. (17 pages)</t>
-        </is>
-      </c>
-      <c r="F6" s="6" t="inlineStr">
-        <is>
-          <t>Done. Counsel to confirm the exact legal form (e.g. "NEMI Corp." vs "NEMI Corporation").</t>
-        </is>
-      </c>
-      <c r="G6" s="6" t="inlineStr">
-        <is>
-          <t>Must match the S-4 entity. The decks name NEMI CORP, US HoldCo (Texas).</t>
-        </is>
-      </c>
-      <c r="H6" s="6" t="inlineStr">
-        <is>
-          <t>Counsel</t>
-        </is>
-      </c>
-      <c r="I6" s="6" t="inlineStr">
-        <is>
-          <t>29</t>
-        </is>
-      </c>
-      <c r="J6" s="6" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="5" t="n">
-        <v>3</v>
-      </c>
-      <c r="B7" s="13" t="inlineStr">
-        <is>
-          <t>Decided 6 Oct</t>
-        </is>
-      </c>
-      <c r="C7" s="5" t="inlineStr">
+      <c r="B5" s="11" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
         <is>
           <t>Invest</t>
         </is>
       </c>
-      <c r="D7" s="5" t="inlineStr">
+      <c r="D5" s="4" t="inlineStr">
         <is>
           <t>Whole page</t>
         </is>
       </c>
-      <c r="E7" s="5" t="inlineStr">
-        <is>
-          <t>Invest in NEMI — Coming soon</t>
-        </is>
-      </c>
-      <c r="F7" s="5" t="inlineStr">
-        <is>
-          <t>Decided 6 Oct: keep "Coming soon". The decks and teaser still invite investors through invest@nemilmm.com, and an investor site exists at invest-reg-d.nemilmm.com. Counsel to confirm the two are consistent (question drafted).</t>
-        </is>
-      </c>
-      <c r="G7" s="5" t="inlineStr">
-        <is>
-          <t>The teaser and decks send investors to invest@nemilmm.com; a public "coming soon" contradicts that.</t>
-        </is>
-      </c>
-      <c r="H7" s="5" t="inlineStr">
-        <is>
-          <t>CEO + counsel</t>
-        </is>
-      </c>
-      <c r="I7" s="5" t="inlineStr">
+      <c r="E5" s="4" t="inlineStr">
+        <is>
+          <t>Invest in NEMI — Coming soon. "Our investment offerings are not open yet. Stay tuned."</t>
+        </is>
+      </c>
+      <c r="F5" s="4" t="inlineStr">
+        <is>
+          <t>Kept as "Coming soon" for now, by decision. When investing opens, point the Invest button to the investor site (https://invest-reg-d.nemilmm.com/) and replace this page.</t>
+        </is>
+      </c>
+      <c r="G5" s="4" t="inlineStr">
+        <is>
+          <t>The decks invite investors through invest@nemilmm.com, so the site and decks say different things until the page opens.</t>
+        </is>
+      </c>
+      <c r="H5" s="4" t="inlineStr">
+        <is>
+          <t>CEO</t>
+        </is>
+      </c>
+      <c r="I5" s="4" t="inlineStr">
         <is>
           <t>23</t>
         </is>
       </c>
-      <c r="J7" s="5" t="inlineStr">
-        <is>
-          <t>Not needed</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="B8" s="9" t="inlineStr">
-        <is>
-          <t>1 · Decide</t>
-        </is>
-      </c>
-      <c r="C8" s="4" t="inlineStr">
-        <is>
-          <t>About</t>
-        </is>
-      </c>
-      <c r="D8" s="4" t="inlineStr">
-        <is>
-          <t>CEO bio</t>
-        </is>
-      </c>
-      <c r="E8" s="4" t="inlineStr">
-        <is>
-          <t>Acquired and expanded NEMI's manufacturing base to over 300,000 sq ft in India.</t>
-        </is>
-      </c>
-      <c r="F8" s="4" t="inlineStr">
-        <is>
-          <t>Site and all three decks now say "built the EV business and acquired and expanded the MaaS factories". CEO or CFO to confirm the history is exact.</t>
-        </is>
-      </c>
-      <c r="G8" s="4" t="inlineStr">
-        <is>
-          <t>"Greenfield" and "acquired" can both be partly true. The site and decks must say the same thing.</t>
-        </is>
-      </c>
-      <c r="H8" s="4" t="inlineStr">
-        <is>
-          <t>CEO + CFO</t>
-        </is>
-      </c>
-      <c r="I8" s="4" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="J8" s="10" t="inlineStr">
-        <is>
-          <t>In progress</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="B9" s="9" t="inlineStr">
-        <is>
-          <t>1 · Decide</t>
-        </is>
-      </c>
-      <c r="C9" s="4" t="inlineStr">
-        <is>
-          <t>About + decks</t>
-        </is>
-      </c>
-      <c r="D9" s="4" t="inlineStr">
-        <is>
-          <t>Kevin Flick bio</t>
-        </is>
-      </c>
-      <c r="E9" s="4" t="inlineStr">
-        <is>
-          <t>Site: Canacol Energy and EY (from his LinkedIn). Decks: "Goldman Sachs · Hicks Muse · $5B+ raised · listed 3 companies".</t>
-        </is>
-      </c>
-      <c r="F9" s="4" t="inlineStr">
-        <is>
-          <t>Message drafted (see "Messages to send"). Site keeps the LinkedIn-based bio until his CV confirms Goldman Sachs and Hicks Muse; the decks were not changed on this point.</t>
-        </is>
-      </c>
-      <c r="G9" s="4" t="inlineStr">
-        <is>
-          <t>An officer bio in the S-4 that differs from investor decks is a disclosure problem.</t>
-        </is>
-      </c>
-      <c r="H9" s="4" t="inlineStr">
-        <is>
-          <t>CFO + counsel</t>
-        </is>
-      </c>
-      <c r="I9" s="4" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="J9" s="10" t="inlineStr">
-        <is>
-          <t>In progress</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="B10" s="9" t="inlineStr">
-        <is>
-          <t>1 · Decide</t>
-        </is>
-      </c>
-      <c r="C10" s="4" t="inlineStr">
-        <is>
-          <t>Teaser (pre-NDA)</t>
-        </is>
-      </c>
-      <c r="D10" s="4" t="inlineStr">
-        <is>
-          <t>Path to listing</t>
-        </is>
-      </c>
-      <c r="E10" s="4" t="inlineStr">
-        <is>
-          <t>The teaser's "path to listing" section, with dates.</t>
-        </is>
-      </c>
-      <c r="F10" s="4" t="inlineStr">
-        <is>
-          <t>Question drafted for counsel (see "Messages to send").</t>
-        </is>
-      </c>
-      <c r="G10" s="4" t="inlineStr">
-        <is>
-          <t>The plan says nothing about the transaction is public before announcement. The teaser is the least controlled document.</t>
-        </is>
-      </c>
-      <c r="H10" s="4" t="inlineStr">
-        <is>
-          <t>Counsel</t>
-        </is>
-      </c>
-      <c r="I10" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J10" s="10" t="inlineStr">
-        <is>
-          <t>In progress</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="4" t="n">
-        <v>7</v>
-      </c>
-      <c r="B11" s="11" t="inlineStr">
-        <is>
-          <t>2 · Decide</t>
-        </is>
-      </c>
-      <c r="C11" s="4" t="inlineStr">
-        <is>
-          <t>About</t>
-        </is>
-      </c>
-      <c r="D11" s="4" t="inlineStr">
-        <is>
-          <t>India finance title and spellings</t>
-        </is>
-      </c>
-      <c r="E11" s="4" t="inlineStr">
-        <is>
-          <t>"Finance Head · India" · "Subramanian Ramaswamy"</t>
-        </is>
-      </c>
-      <c r="F11" s="4" t="inlineStr">
-        <is>
-          <t>Site keeps "Finance Head · India"; vPresent copy corrected to match. Spelling question drafted for him (see "Messages to send").</t>
-        </is>
-      </c>
-      <c r="G11" s="4" t="inlineStr">
-        <is>
-          <t>Names and titles must match the filing.</t>
-        </is>
-      </c>
-      <c r="H11" s="4" t="inlineStr">
-        <is>
-          <t>HR + counsel</t>
-        </is>
-      </c>
-      <c r="I11" s="4" t="inlineStr">
-        <is>
-          <t>26</t>
-        </is>
-      </c>
-      <c r="J11" s="10" t="inlineStr">
-        <is>
-          <t>In progress</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="4" t="n">
-        <v>8</v>
-      </c>
-      <c r="B12" s="11" t="inlineStr">
-        <is>
-          <t>2 · Decide</t>
-        </is>
-      </c>
-      <c r="C12" s="4" t="inlineStr">
-        <is>
-          <t>Case Messenger · Case Studies</t>
-        </is>
-      </c>
-      <c r="D12" s="4" t="inlineStr">
-        <is>
-          <t>BNC program cost</t>
-        </is>
-      </c>
-      <c r="E12" s="4" t="inlineStr">
-        <is>
-          <t>"under $1M"</t>
-        </is>
-      </c>
-      <c r="F12" s="4" t="inlineStr">
-        <is>
-          <t>Site now says under $0.5M, as every deck does. CFO to confirm against the ledger (message drafted).</t>
-        </is>
-      </c>
-      <c r="G12" s="4" t="inlineStr">
-        <is>
-          <t>Precision, not a contradiction.</t>
-        </is>
-      </c>
-      <c r="H12" s="4" t="inlineStr">
-        <is>
-          <t>CFO</t>
-        </is>
-      </c>
-      <c r="I12" s="4" t="inlineStr">
-        <is>
-          <t>11</t>
-        </is>
-      </c>
-      <c r="J12" s="10" t="inlineStr">
-        <is>
-          <t>In progress</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="4" t="n">
-        <v>9</v>
-      </c>
-      <c r="B13" s="11" t="inlineStr">
-        <is>
-          <t>2 · Decide</t>
-        </is>
-      </c>
-      <c r="C13" s="4" t="inlineStr">
-        <is>
-          <t>About</t>
-        </is>
-      </c>
-      <c r="D13" s="4" t="inlineStr">
-        <is>
-          <t>Advisory bench</t>
-        </is>
-      </c>
-      <c r="E13" s="4" t="inlineStr">
-        <is>
-          <t>Advisor titles: Board Advisor · Chairman · AxisCades · Ex-CEO · Ashok Leyland · Ex-Sr Partner · McKinsey</t>
-        </is>
-      </c>
-      <c r="F13" s="4" t="inlineStr">
-        <is>
-          <t>Message drafted for the CEO (see "Messages to send").</t>
-        </is>
-      </c>
-      <c r="G13" s="4" t="inlineStr">
-        <is>
-          <t>The S-4 lists these exactly.</t>
-        </is>
-      </c>
-      <c r="H13" s="4" t="inlineStr">
-        <is>
-          <t>CEO + counsel</t>
-        </is>
-      </c>
-      <c r="I13" s="4" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="J13" s="10" t="inlineStr">
-        <is>
-          <t>In progress</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="4" t="n">
-        <v>10</v>
-      </c>
-      <c r="B14" s="11" t="inlineStr">
-        <is>
-          <t>2 · Decide</t>
-        </is>
-      </c>
-      <c r="C14" s="4" t="inlineStr">
-        <is>
-          <t>About</t>
-        </is>
-      </c>
-      <c r="D14" s="4" t="inlineStr">
-        <is>
-          <t>Gokul Madhavan bio</t>
-        </is>
-      </c>
-      <c r="E14" s="4" t="inlineStr">
-        <is>
-          <t>Interim strategy wording plus degrees.</t>
-        </is>
-      </c>
-      <c r="F14" s="4" t="inlineStr">
-        <is>
-          <t>Message drafted (see "Messages to send").</t>
-        </is>
-      </c>
-      <c r="G14" s="4" t="inlineStr">
-        <is>
-          <t>Interim text, noted in the page.</t>
-        </is>
-      </c>
-      <c r="H14" s="4" t="inlineStr">
-        <is>
-          <t>CSO</t>
-        </is>
-      </c>
-      <c r="I14" s="4" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="J14" s="10" t="inlineStr">
-        <is>
-          <t>In progress</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="4" t="n">
-        <v>11</v>
-      </c>
-      <c r="B15" s="12" t="inlineStr">
-        <is>
-          <t>3 · Evidence</t>
-        </is>
-      </c>
-      <c r="C15" s="4" t="inlineStr">
-        <is>
-          <t>Case Messenger (BNC)</t>
-        </is>
-      </c>
-      <c r="D15" s="4" t="inlineStr">
-        <is>
-          <t>Results</t>
-        </is>
-      </c>
-      <c r="E15" s="4" t="inlineStr">
-        <is>
-          <t>18 → 9 months, 100% spec met, sub-$1,000 price point</t>
-        </is>
-      </c>
-      <c r="F15" s="4" t="inlineStr">
-        <is>
-          <t>Project plan, test report and BOM costing on file, or remove.</t>
-        </is>
-      </c>
-      <c r="G15" s="4" t="inlineStr">
-        <is>
-          <t>Every number traces to a document.</t>
-        </is>
-      </c>
-      <c r="H15" s="4" t="inlineStr">
-        <is>
-          <t>COO</t>
-        </is>
-      </c>
-      <c r="I15" s="4" t="inlineStr">
-        <is>
-          <t>12</t>
-        </is>
-      </c>
-      <c r="J15" s="10" t="inlineStr">
+      <c r="J5" s="12" t="inlineStr">
         <is>
           <t>To do</t>
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="4" t="n">
-        <v>12</v>
-      </c>
-      <c r="B16" s="12" t="inlineStr">
-        <is>
-          <t>3 · Evidence</t>
-        </is>
-      </c>
-      <c r="C16" s="4" t="inlineStr">
-        <is>
-          <t>Case Coffee</t>
-        </is>
-      </c>
-      <c r="D16" s="4" t="inlineStr">
-        <is>
-          <t>Results</t>
-        </is>
-      </c>
-      <c r="E16" s="4" t="inlineStr">
-        <is>
-          <t>12+ → 5 weeks, ~$100k, −20% BOM, 400 a month</t>
-        </is>
-      </c>
-      <c r="F16" s="4" t="inlineStr">
-        <is>
-          <t>Customer's written consent to use their data, or remove.</t>
-        </is>
-      </c>
-      <c r="G16" s="4" t="inlineStr">
-        <is>
-          <t>Rests on the customer's quotes.</t>
-        </is>
-      </c>
-      <c r="H16" s="4" t="inlineStr">
-        <is>
-          <t>Sales + CFO</t>
-        </is>
-      </c>
-      <c r="I16" s="4" t="inlineStr">
-        <is>
-          <t>13</t>
-        </is>
-      </c>
-      <c r="J16" s="10" t="inlineStr">
-        <is>
-          <t>To do</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="4" t="n">
-        <v>13</v>
-      </c>
-      <c r="B17" s="12" t="inlineStr">
-        <is>
-          <t>3 · Evidence</t>
-        </is>
-      </c>
-      <c r="C17" s="4" t="inlineStr">
-        <is>
-          <t>Case Drone · Case Studies</t>
-        </is>
-      </c>
-      <c r="D17" s="4" t="inlineStr">
-        <is>
-          <t>Results</t>
-        </is>
-      </c>
-      <c r="E17" s="4" t="inlineStr">
-        <is>
-          <t>16 → 4 months, $100k, 4/4 in-house, −20% BOM, "4× faster"</t>
-        </is>
-      </c>
-      <c r="F17" s="4" t="inlineStr">
-        <is>
-          <t>Evidence pack. These figures match the decks.</t>
-        </is>
-      </c>
-      <c r="G17" s="4" t="inlineStr">
-        <is>
-          <t>Only partly evidenced.</t>
-        </is>
-      </c>
-      <c r="H17" s="4" t="inlineStr">
-        <is>
-          <t>CFO</t>
-        </is>
-      </c>
-      <c r="I17" s="4" t="inlineStr">
-        <is>
-          <t>14</t>
-        </is>
-      </c>
-      <c r="J17" s="10" t="inlineStr">
-        <is>
-          <t>To do</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="4" t="n">
-        <v>14</v>
-      </c>
-      <c r="B18" s="12" t="inlineStr">
-        <is>
-          <t>3 · Evidence</t>
-        </is>
-      </c>
-      <c r="C18" s="4" t="inlineStr">
-        <is>
-          <t>Case PMI · Case Studies</t>
-        </is>
-      </c>
-      <c r="D18" s="4" t="inlineStr">
-        <is>
-          <t>Results</t>
-        </is>
-      </c>
-      <c r="E18" s="4" t="inlineStr">
-        <is>
-          <t>7 → 3 hrs, ~15 a day, 10–15 µm, under a week, "3–4× tighter"</t>
-        </is>
-      </c>
-      <c r="F18" s="4" t="inlineStr">
-        <is>
-          <t>Machine logs and CMM records on file.</t>
-        </is>
-      </c>
-      <c r="G18" s="4" t="inlineStr">
-        <is>
-          <t>Performance claims need records.</t>
-        </is>
-      </c>
-      <c r="H18" s="4" t="inlineStr">
-        <is>
-          <t>COO</t>
-        </is>
-      </c>
-      <c r="I18" s="4" t="inlineStr">
-        <is>
-          <t>15</t>
-        </is>
-      </c>
-      <c r="J18" s="10" t="inlineStr">
-        <is>
-          <t>To do</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="4" t="n">
-        <v>15</v>
-      </c>
-      <c r="B19" s="12" t="inlineStr">
-        <is>
-          <t>3 · Evidence</t>
-        </is>
-      </c>
-      <c r="C19" s="4" t="inlineStr">
-        <is>
-          <t>Case Drone</t>
-        </is>
-      </c>
-      <c r="D19" s="4" t="inlineStr">
-        <is>
-          <t>Hero image</t>
-        </is>
-      </c>
-      <c r="E19" s="4" t="inlineStr">
-        <is>
-          <t>Labelled "Illustration".</t>
-        </is>
-      </c>
-      <c r="F19" s="4" t="inlineStr">
-        <is>
-          <t>Confirm it is not the customer's airframe; if it is, get consent or replace.</t>
-        </is>
-      </c>
-      <c r="G19" s="4" t="inlineStr">
-        <is>
-          <t>Customer property.</t>
-        </is>
-      </c>
-      <c r="H19" s="4" t="inlineStr">
-        <is>
-          <t>CEO</t>
-        </is>
-      </c>
-      <c r="I19" s="4" t="inlineStr">
-        <is>
-          <t>9</t>
-        </is>
-      </c>
-      <c r="J19" s="10" t="inlineStr">
-        <is>
-          <t>To do</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="4" t="n">
-        <v>16</v>
-      </c>
-      <c r="B20" s="12" t="inlineStr">
-        <is>
-          <t>3 · Evidence</t>
-        </is>
-      </c>
-      <c r="C20" s="4" t="inlineStr">
-        <is>
-          <t>FAQ · badges</t>
-        </is>
-      </c>
-      <c r="D20" s="4" t="inlineStr">
-        <is>
-          <t>Certifications</t>
-        </is>
-      </c>
-      <c r="E20" s="4" t="inlineStr">
-        <is>
-          <t>AS9100D:2016 and ISO 9001:2015 "our factories"</t>
-        </is>
-      </c>
-      <c r="F20" s="4" t="inlineStr">
-        <is>
-          <t>Name the certified entity and sites from the certificates.</t>
-        </is>
-      </c>
-      <c r="G20" s="4" t="inlineStr">
-        <is>
-          <t>Scope must cover every named site.</t>
-        </is>
-      </c>
-      <c r="H20" s="4" t="inlineStr">
-        <is>
-          <t>Quality</t>
-        </is>
-      </c>
-      <c r="I20" s="4" t="inlineStr">
-        <is>
-          <t>16</t>
-        </is>
-      </c>
-      <c r="J20" s="10" t="inlineStr">
-        <is>
-          <t>To do</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="4" t="n">
-        <v>17</v>
-      </c>
-      <c r="B21" s="12" t="inlineStr">
-        <is>
-          <t>3 · Evidence</t>
-        </is>
-      </c>
-      <c r="C21" s="4" t="inlineStr">
-        <is>
-          <t>Home</t>
-        </is>
-      </c>
-      <c r="D21" s="4" t="inlineStr">
-        <is>
-          <t>Market images, BOSS E-TWIN, app screenshots</t>
-        </is>
-      </c>
-      <c r="E21" s="4" t="inlineStr">
-        <is>
-          <t>Third-party market photos · group brand without a label · Anvil/Orion/Atlas screens</t>
-        </is>
-      </c>
-      <c r="F21" s="4" t="inlineStr">
-        <is>
-          <t>Licence or replace the photos; label E-TWIN as internal; confirm screens are the real product.</t>
-        </is>
-      </c>
-      <c r="G21" s="4" t="inlineStr">
-        <is>
-          <t>Implied customers and implied shipped software.</t>
-        </is>
-      </c>
-      <c r="H21" s="4" t="inlineStr">
-        <is>
-          <t>CEO + CTO + Marketing</t>
-        </is>
-      </c>
-      <c r="I21" s="4" t="inlineStr">
-        <is>
-          <t>21, 22, 34, 35</t>
-        </is>
-      </c>
-      <c r="J21" s="10" t="inlineStr">
-        <is>
-          <t>To do</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="4" t="n">
-        <v>18</v>
-      </c>
-      <c r="B22" s="12" t="inlineStr">
-        <is>
-          <t>3 · Evidence</t>
-        </is>
-      </c>
-      <c r="C22" s="4" t="inlineStr">
-        <is>
-          <t>About · Home · Offerings</t>
-        </is>
-      </c>
-      <c r="D22" s="4" t="inlineStr">
-        <is>
-          <t>Archive photos and videos</t>
-        </is>
-      </c>
-      <c r="E22" s="4" t="inlineStr">
-        <is>
-          <t>Eras photos (1913, 1950, 1980) · 14 videos</t>
-        </is>
-      </c>
-      <c r="F22" s="4" t="inlineStr">
-        <is>
-          <t>Record source and licence for each.</t>
-        </is>
-      </c>
-      <c r="G22" s="4" t="inlineStr">
-        <is>
-          <t>Third-party media needs a licence on file.</t>
-        </is>
-      </c>
-      <c r="H22" s="4" t="inlineStr">
-        <is>
-          <t>Marketing</t>
-        </is>
-      </c>
-      <c r="I22" s="4" t="inlineStr">
-        <is>
-          <t>27, 42</t>
-        </is>
-      </c>
-      <c r="J22" s="10" t="inlineStr">
-        <is>
-          <t>To do</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="4" t="n">
-        <v>19</v>
-      </c>
-      <c r="B23" s="12" t="inlineStr">
-        <is>
-          <t>3 · Evidence</t>
-        </is>
-      </c>
-      <c r="C23" s="4" t="inlineStr">
-        <is>
-          <t>Decks and teaser</t>
-        </is>
-      </c>
-      <c r="D23" s="4" t="inlineStr">
-        <is>
-          <t>Numbers not on the site</t>
-        </is>
-      </c>
-      <c r="E23" s="4" t="inlineStr">
-        <is>
-          <t>Customer count, retention, productivity, "owned factories", "built greenfield"</t>
-        </is>
-      </c>
-      <c r="F23" s="4" t="inlineStr">
-        <is>
-          <t>Make sure each has a document behind it before anything is filed; check "owned" against leases and deeds.</t>
-        </is>
-      </c>
-      <c r="G23" s="4" t="inlineStr">
-        <is>
-          <t>The S-4 is written from the same facts.</t>
-        </is>
-      </c>
-      <c r="H23" s="4" t="inlineStr">
-        <is>
-          <t>CFO + Marketing</t>
-        </is>
-      </c>
-      <c r="I23" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J23" s="10" t="inlineStr">
-        <is>
-          <t>To do</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="4" t="n">
-        <v>20</v>
-      </c>
-      <c r="B24" s="7" t="inlineStr">
-        <is>
-          <t>Done 5 Oct</t>
-        </is>
-      </c>
-      <c r="C24" s="4" t="inlineStr">
-        <is>
-          <t>Case Drone</t>
-        </is>
-      </c>
-      <c r="D24" s="4" t="inlineStr">
-        <is>
-          <t>Broken sentences and empty table cell</t>
-        </is>
-      </c>
-      <c r="E24" s="4" t="inlineStr">
-        <is>
-          <t>Fixed — see Corrections tab.</t>
-        </is>
-      </c>
-      <c r="F24" s="4" t="n"/>
-      <c r="G24" s="4" t="n"/>
-      <c r="H24" s="4" t="n"/>
-      <c r="I24" s="4" t="inlineStr">
-        <is>
-          <t>14</t>
-        </is>
-      </c>
-      <c r="J24" s="10" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="4" t="n">
-        <v>21</v>
-      </c>
-      <c r="B25" s="7" t="inlineStr">
-        <is>
-          <t>Done 5 Oct</t>
-        </is>
-      </c>
-      <c r="C25" s="4" t="inlineStr">
-        <is>
-          <t>FAQ · Contact</t>
-        </is>
-      </c>
-      <c r="D25" s="4" t="inlineStr">
-        <is>
-          <t>Broken sentence, empty element</t>
-        </is>
-      </c>
-      <c r="E25" s="4" t="inlineStr">
-        <is>
-          <t>Fixed.</t>
-        </is>
-      </c>
-      <c r="F25" s="4" t="n"/>
-      <c r="G25" s="4" t="n"/>
-      <c r="H25" s="4" t="n"/>
-      <c r="I25" s="4" t="inlineStr">
-        <is>
-          <t>25</t>
-        </is>
-      </c>
-      <c r="J25" s="10" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="4" t="n">
-        <v>22</v>
-      </c>
-      <c r="B26" s="7" t="inlineStr">
-        <is>
-          <t>Done 5 Oct</t>
-        </is>
-      </c>
-      <c r="C26" s="4" t="inlineStr">
-        <is>
-          <t>Case Studies · Case Coffee</t>
-        </is>
-      </c>
-      <c r="D26" s="4" t="inlineStr">
-        <is>
-          <t>"Typical" tag, "Benchmark withheld"</t>
-        </is>
-      </c>
-      <c r="E26" s="4" t="inlineStr">
-        <is>
-          <t>Removed / replaced with "—".</t>
-        </is>
-      </c>
-      <c r="F26" s="4" t="n"/>
-      <c r="G26" s="4" t="n"/>
-      <c r="H26" s="4" t="n"/>
-      <c r="I26" s="4" t="inlineStr">
-        <is>
-          <t>11, 13</t>
-        </is>
-      </c>
-      <c r="J26" s="10" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="4" t="n">
-        <v>23</v>
-      </c>
-      <c r="B27" s="7" t="inlineStr">
-        <is>
-          <t>Done 5 Oct</t>
-        </is>
-      </c>
-      <c r="C27" s="4" t="inlineStr">
-        <is>
-          <t>LMM Stack</t>
-        </is>
-      </c>
-      <c r="D27" s="4" t="inlineStr">
-        <is>
-          <t>"and profits on its own"</t>
-        </is>
-      </c>
-      <c r="E27" s="4" t="inlineStr">
-        <is>
-          <t>Removed.</t>
-        </is>
-      </c>
-      <c r="F27" s="4" t="n"/>
-      <c r="G27" s="4" t="n"/>
-      <c r="H27" s="4" t="n"/>
-      <c r="I27" s="4" t="inlineStr">
-        <is>
-          <t>5, 20</t>
-        </is>
-      </c>
-      <c r="J27" s="10" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="4" t="n">
-        <v>24</v>
-      </c>
-      <c r="B28" s="7" t="inlineStr">
-        <is>
-          <t>Done 5 Oct</t>
-        </is>
-      </c>
-      <c r="C28" s="4" t="inlineStr">
-        <is>
-          <t>About · Offerings · Home</t>
-        </is>
-      </c>
-      <c r="D28" s="4" t="inlineStr">
-        <is>
-          <t>Five "proven"</t>
-        </is>
-      </c>
-      <c r="E28" s="4" t="inlineStr">
-        <is>
-          <t>Replaced with "run", "tested", "in use with".</t>
-        </is>
-      </c>
-      <c r="F28" s="4" t="n"/>
-      <c r="G28" s="4" t="n"/>
-      <c r="H28" s="4" t="n"/>
-      <c r="I28" s="4" t="inlineStr">
-        <is>
-          <t>17, 31</t>
-        </is>
-      </c>
-      <c r="J28" s="10" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="4" t="n">
-        <v>25</v>
-      </c>
-      <c r="B29" s="7" t="inlineStr">
-        <is>
-          <t>Done 5 Oct</t>
-        </is>
-      </c>
-      <c r="C29" s="4" t="inlineStr">
-        <is>
-          <t>Home</t>
-        </is>
-      </c>
-      <c r="D29" s="4" t="inlineStr">
-        <is>
-          <t>App status badges</t>
-        </is>
-      </c>
-      <c r="E29" s="4" t="inlineStr">
-        <is>
-          <t>Anvil Live · Orion In validation · Atlas Roadmap.</t>
-        </is>
-      </c>
-      <c r="F29" s="4" t="n"/>
-      <c r="G29" s="4" t="n"/>
-      <c r="H29" s="4" t="n"/>
-      <c r="I29" s="4" t="inlineStr">
-        <is>
-          <t>19</t>
-        </is>
-      </c>
-      <c r="J29" s="10" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="4" t="n">
-        <v>26</v>
-      </c>
-      <c r="B30" s="7" t="inlineStr">
-        <is>
-          <t>Done 5 Oct</t>
-        </is>
-      </c>
-      <c r="C30" s="4" t="inlineStr">
-        <is>
-          <t>About</t>
-        </is>
-      </c>
-      <c r="D30" s="4" t="inlineStr">
-        <is>
-          <t>Team facts and titles</t>
-        </is>
-      </c>
-      <c r="E30" s="4" t="inlineStr">
-        <is>
-          <t>Degrees and employers restored; President titles back; Ravi Narayanan; unsourced additions removed.</t>
-        </is>
-      </c>
-      <c r="F30" s="4" t="n"/>
-      <c r="G30" s="4" t="n"/>
-      <c r="H30" s="4" t="n"/>
-      <c r="I30" s="4" t="inlineStr">
-        <is>
-          <t>3, 26</t>
-        </is>
-      </c>
-      <c r="J30" s="10" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="4" t="n">
-        <v>27</v>
-      </c>
-      <c r="B31" s="7" t="inlineStr">
-        <is>
-          <t>Done 5 Oct</t>
-        </is>
-      </c>
-      <c r="C31" s="4" t="inlineStr">
-        <is>
-          <t>Home · Careers · FAQ · Case pages · Offerings</t>
-        </is>
-      </c>
-      <c r="D31" s="4" t="inlineStr">
-        <is>
-          <t>Polish</t>
-        </is>
-      </c>
-      <c r="E31" s="4" t="inlineStr">
-        <is>
-          <t>Hero line, Careers line, reply, program, Test-bed EV.</t>
-        </is>
-      </c>
-      <c r="F31" s="4" t="n"/>
-      <c r="G31" s="4" t="n"/>
-      <c r="H31" s="4" t="n"/>
-      <c r="I31" s="4" t="inlineStr">
-        <is>
-          <t>10, 30</t>
-        </is>
-      </c>
-      <c r="J31" s="10" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="4" t="n">
-        <v>28</v>
-      </c>
-      <c r="B32" s="13" t="inlineStr">
-        <is>
-          <t>Not needed</t>
-        </is>
-      </c>
-      <c r="C32" s="4" t="inlineStr">
-        <is>
-          <t>LMM Stack · About</t>
-        </is>
-      </c>
-      <c r="D32" s="4" t="inlineStr">
-        <is>
-          <t>Footprint note "expansion planned"</t>
-        </is>
-      </c>
-      <c r="E32" s="4" t="inlineStr">
-        <is>
-          <t>Left out: it is a forward-looking line, the reason "more locations coming soon" was removed.</t>
-        </is>
-      </c>
-      <c r="F32" s="4" t="n"/>
-      <c r="G32" s="4" t="n"/>
-      <c r="H32" s="4" t="n"/>
-      <c r="I32" s="4" t="inlineStr">
-        <is>
-          <t>25</t>
-        </is>
-      </c>
-      <c r="J32" s="10" t="inlineStr">
-        <is>
-          <t>Not needed</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="4" t="n">
-        <v>29</v>
-      </c>
-      <c r="B33" s="13" t="inlineStr">
-        <is>
-          <t>Not needed</t>
-        </is>
-      </c>
-      <c r="C33" s="4" t="inlineStr">
-        <is>
-          <t>About · Master Plan</t>
-        </is>
-      </c>
-      <c r="D33" s="4" t="inlineStr">
-        <is>
-          <t>Phase names in the deck's words</t>
-        </is>
-      </c>
-      <c r="E33" s="4" t="inlineStr">
-        <is>
-          <t>Left as the founder's letter words them.</t>
-        </is>
-      </c>
-      <c r="F33" s="4" t="n"/>
-      <c r="G33" s="4" t="n"/>
-      <c r="H33" s="4" t="n"/>
-      <c r="I33" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J33" s="10" t="inlineStr">
-        <is>
-          <t>Not needed</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A4:J33"/>
+  <autoFilter ref="A4:J5"/>
   <conditionalFormatting sqref="A5:J33">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>$J5="Done"</formula>
@@ -5506,185 +4823,4 @@
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:D10"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="5" customWidth="1" min="1" max="1"/>
-    <col width="22" customWidth="1" min="2" max="2"/>
-    <col width="34" customWidth="1" min="3" max="3"/>
-    <col width="110" customWidth="1" min="4" max="4"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Messages to send: the items only a person can close</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>Copy, adjust and send. Each one closes an open row on "Still to update".</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="14" t="inlineStr">
-        <is>
-          <t>#</t>
-        </is>
-      </c>
-      <c r="B4" s="14" t="inlineStr">
-        <is>
-          <t>To</t>
-        </is>
-      </c>
-      <c r="C4" s="14" t="inlineStr">
-        <is>
-          <t>Subject</t>
-        </is>
-      </c>
-      <c r="D4" s="14" t="inlineStr">
-        <is>
-          <t>Message</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="15" t="n">
-        <v>1</v>
-      </c>
-      <c r="B5" s="15" t="inlineStr">
-        <is>
-          <t>US securities counsel</t>
-        </is>
-      </c>
-      <c r="C5" s="15" t="inlineStr">
-        <is>
-          <t>Five questions before BCA signing</t>
-        </is>
-      </c>
-      <c r="D5" s="15" t="inlineStr">
-        <is>
-          <t>1. Our pre-NDA investor teaser describes the transaction process with dates. Can a pre-NDA document carry that before announcement, or should it come out?
-2. The website footer now reads "© 2026 NEMI Corp." Please confirm the exact legal name the S-4 will use.
-3. The founder's letter on the website says "MaaS is profitable on its own" and "profitably, today". The group is not profitable; the MaaS segment is EBITDA-positive on management figures. Should the letter state the segment measure, or should the lines come out?
-4. The website's Invest page says "Coming soon", while our decks and teaser invite investors through invest@nemilmm.com, and an investor site exists at invest-reg-d.nemilmm.com. Is that consistent, or should one of them change?
-5. Two advisors and a director may need relationship disclosures. Please advise what the S-4 requires.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="15" t="n">
-        <v>2</v>
-      </c>
-      <c r="B6" s="15" t="inlineStr">
-        <is>
-          <t>Kevin Flick</t>
-        </is>
-      </c>
-      <c r="C6" s="15" t="inlineStr">
-        <is>
-          <t>Your bio for the website and the S-4</t>
-        </is>
-      </c>
-      <c r="D6" s="15" t="inlineStr">
-        <is>
-          <t>Kevin, our decks describe you as "Goldman Sachs · Hicks Muse · $5B+ raised · listed 3 companies on NASDAQ, NYSE and TSX". The website uses a shorter bio based on your LinkedIn (Canacol Energy, EY). Could you send your CV or confirm the exact wording you want used, and sign off on it? It needs to match the S-4 word for word.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="15" t="n">
-        <v>3</v>
-      </c>
-      <c r="B7" s="15" t="inlineStr">
-        <is>
-          <t>Subramanian</t>
-        </is>
-      </c>
-      <c r="C7" s="15" t="inlineStr">
-        <is>
-          <t>Your title and the spelling of your name</t>
-        </is>
-      </c>
-      <c r="D7" s="15" t="inlineStr">
-        <is>
-          <t>Our decks spell your name "Ramasamy" and the website "Ramaswamy". Which is correct? Your title on the website is "Finance Head · India", so it does not read as a second CFO in the officer list. Are you happy with that?</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="15" t="n">
-        <v>4</v>
-      </c>
-      <c r="B8" s="15" t="inlineStr">
-        <is>
-          <t>Gokul Madhavan</t>
-        </is>
-      </c>
-      <c r="C8" s="15" t="inlineStr">
-        <is>
-          <t>Your bio</t>
-        </is>
-      </c>
-      <c r="D8" s="15" t="inlineStr">
-        <is>
-          <t>The website carries an interim bio for your strategy role: "Corporate development and transformation. M&amp;A integration, digital finance operations, and the work of turning strategy into operating plans across the group. PhD Harvard, MBA Yale." Please send the wording you want, so it can match the S-4.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="15" t="n">
-        <v>5</v>
-      </c>
-      <c r="B9" s="15" t="inlineStr">
-        <is>
-          <t>CFO</t>
-        </is>
-      </c>
-      <c r="C9" s="15" t="inlineStr">
-        <is>
-          <t>Two figures to confirm</t>
-        </is>
-      </c>
-      <c r="D9" s="15" t="inlineStr">
-        <is>
-          <t>1. BNC Messenger program cost: the website and decks now say "under $0.5M". Please confirm against the ledger.
-2. The CEO bio now reads "Built NEMI's EV business and acquired and expanded its MaaS factories, now over 300,000 sq ft in India." Please confirm the history and the square footage against the leases and deeds.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="15" t="n">
-        <v>6</v>
-      </c>
-      <c r="B10" s="15" t="inlineStr">
-        <is>
-          <t>CEO</t>
-        </is>
-      </c>
-      <c r="C10" s="15" t="inlineStr">
-        <is>
-          <t>Advisors and board</t>
-        </is>
-      </c>
-      <c r="D10" s="15" t="inlineStr">
-        <is>
-          <t>Please confirm each advisor's seat and title as shown on the website (Board Advisor; Chairman · AxisCades; Ex-CEO · Ashok Leyland; Ex-Sr Partner · McKinsey), and flag any family relationship with a director or officer, so counsel can disclose it.</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
Change log: X link row
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018MafBKjuv7rZ7cieL7GV7x
</commit_message>
<xml_diff>
--- a/_s4/NEMI_BCA-Ready_all_changes.xlsx
+++ b/_s4/NEMI_BCA-Ready_all_changes.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Still to update" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'All changes'!$A$4:$J$87</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'All changes'!$A$4:$J$88</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Still to update'!$A$4:$J$5</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -535,7 +535,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J87"/>
+  <dimension ref="A1:J88"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -560,7 +560,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>6 Oct 2026. 83 rows, everything done or decided to date. 50 make BCA-Ready differ from the live site; 20 were made and later undone, so that part matches the live site again; 13 were checked and kept as they are. Source of truth for facts: vShare and vPresent (Oct 2026). Grey = live wording · Green = BCA-Ready wording. List # = item in the website update list.</t>
+          <t>6 Oct 2026. 84 rows, everything done or decided to date. 51 make BCA-Ready differ from the live site; 20 were made and later undone, so that part matches the live site again; 13 were checked and kept as they are. Source of truth for facts: vShare and vPresent (Oct 2026). Grey = live wording · Green = BCA-Ready wording. List # = item in the website update list.</t>
         </is>
       </c>
     </row>
@@ -4666,8 +4666,54 @@
       </c>
       <c r="J87" s="4" t="inlineStr"/>
     </row>
+    <row r="88">
+      <c r="A88" s="4" t="n">
+        <v>84</v>
+      </c>
+      <c r="B88" s="4" t="inlineStr">
+        <is>
+          <t>All pages</t>
+        </is>
+      </c>
+      <c r="C88" s="4" t="inlineStr">
+        <is>
+          <t>Footer X link and share-card handle</t>
+        </is>
+      </c>
+      <c r="D88" s="5" t="inlineStr">
+        <is>
+          <t>Link: https://x.com/Nemi_LMM · Handle: @Nemi_LMM</t>
+        </is>
+      </c>
+      <c r="E88" s="6" t="inlineStr">
+        <is>
+          <t>Link: https://x.com/Nemi_corp · Handle: @Nemi_corp</t>
+        </is>
+      </c>
+      <c r="F88" s="4" t="inlineStr">
+        <is>
+          <t>X account changed on every page (18 links, 17 share tags).</t>
+        </is>
+      </c>
+      <c r="G88" s="4" t="inlineStr">
+        <is>
+          <t>The company's X account is Nemi Corp (@Nemi_corp).</t>
+        </is>
+      </c>
+      <c r="H88" s="4" t="inlineStr">
+        <is>
+          <t>6 Oct</t>
+        </is>
+      </c>
+      <c r="I88" s="7" t="inlineStr">
+        <is>
+          <t>In BCA-Ready</t>
+        </is>
+      </c>
+      <c r="J88" s="4" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:J87"/>
+  <autoFilter ref="A4:J88"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Investor Relations draft: banner, intro, presentation, press, leadership, board
Rebuilt to the requested layout, top to bottom:
- banner photo of the factory campus with "Investor Relations"
- intro: what NEMI is building, in the decks' words, no figures
- investor presentation: a cover in the style of the vPresent title slide
  ("LMM for Physical AI", October 2026) and "Request the presentation", which
  goes to invest@nemilmm.com. The deck itself is not added: this repository is
  public and vPresent is under NDA.
- latest press: the World Order post, the Master Plan, and a slot where press
  releases will be listed
- Leadership team and Board of directors as separate sections, using the
  same cards as the About page

Still unpublished: noindex and blocked from serving until announcement day.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018MafBKjuv7rZ7cieL7GV7x
</commit_message>
<xml_diff>
--- a/_s4/NEMI_BCA-Ready_all_changes.xlsx
+++ b/_s4/NEMI_BCA-Ready_all_changes.xlsx
@@ -4733,17 +4733,17 @@
       </c>
       <c r="E89" s="6" t="inlineStr">
         <is>
-          <t>Laid out after agilityrobotics.com/investors: announcement, four quick links (press release, investor presentation, webcast, SEC filings), documents and filings, webcast, questions, team in tabs (Leadership · Board · India operations · Advisors) as photo cards with a "+" that opens each person's background, IR contact, legends.</t>
+          <t>Investor Relations page in this order: banner photo (factory campus) with "Investor Relations"; intro; investor presentation (cover in the style of the vPresent title slide, "Request the presentation" to invest@nemilmm.com); latest press (World Order post, Master Plan, slot for press releases); Leadership team and Board of directors as two separate sections in the About page card format.</t>
         </is>
       </c>
       <c r="F89" s="4" t="inlineStr">
         <is>
-          <t>Page styled for the first time (its layout classes had no styles); team section and quick links added; new 5:4 portrait photos in assets/team/portrait.</t>
+          <t>Rebuilt on 9 Oct to the layout you asked for. vPresent itself is not put on the page or in the repository: the repository is public and the deck is under NDA.</t>
         </is>
       </c>
       <c r="G89" s="4" t="inlineStr">
         <is>
-          <t>Stage 2 of the website plan: the Investors page is built unpublished and switched on at announcement. Deal details stay as {{placeholders}} until the filed press release exists. Team names, titles and bios match the About page and the decks.</t>
+          <t>Stays unpublished (noindex, blocked from serving) until announcement day. Team names, titles and bios match the About page and the decks.</t>
         </is>
       </c>
       <c r="H89" s="4" t="inlineStr">

</xml_diff>